<commit_message>
refactor(config): centralize hardcoded timeout values into config.py
</commit_message>
<xml_diff>
--- a/data/test_data.xlsx
+++ b/data/test_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\TANG_KINH_CAC\PracticeSpace\playwright-automationexercise\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30F477A6-92FE-4D67-9320-E8385E2ADD2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48BE1EDE-C4E3-4383-B8DF-EBDF88B50C32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RegisterData" sheetId="1" r:id="rId1"/>
@@ -461,7 +461,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -540,12 +540,6 @@
     </xf>
     <xf numFmtId="49" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -38106,8 +38100,8 @@
       <c r="R1" s="24"/>
     </row>
     <row r="2" spans="1:18" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A2" s="27" t="s">
-        <v>27</v>
+      <c r="A2" s="25" t="s">
+        <v>9</v>
       </c>
       <c r="B2" s="27" t="s">
         <v>79</v>
@@ -38122,11 +38116,11 @@
         <v>9</v>
       </c>
       <c r="F2" s="24"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="30"/>
-      <c r="I2" s="30"/>
-      <c r="J2" s="30"/>
-      <c r="K2" s="30"/>
+      <c r="G2" s="13"/>
+      <c r="H2" s="14"/>
+      <c r="I2" s="14"/>
+      <c r="J2" s="14"/>
+      <c r="K2" s="14"/>
       <c r="L2" s="24"/>
       <c r="M2" s="24"/>
       <c r="N2" s="24"/>
@@ -38136,8 +38130,8 @@
       <c r="R2" s="24"/>
     </row>
     <row r="3" spans="1:18" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A3" s="27" t="s">
-        <v>27</v>
+      <c r="A3" s="25" t="s">
+        <v>9</v>
       </c>
       <c r="B3" s="27" t="s">
         <v>80</v>
@@ -38152,11 +38146,11 @@
         <v>9</v>
       </c>
       <c r="F3" s="24"/>
-      <c r="G3" s="29"/>
-      <c r="H3" s="30"/>
-      <c r="I3" s="30"/>
-      <c r="J3" s="30"/>
-      <c r="K3" s="30"/>
+      <c r="G3" s="13"/>
+      <c r="H3" s="14"/>
+      <c r="I3" s="14"/>
+      <c r="J3" s="14"/>
+      <c r="K3" s="14"/>
       <c r="L3" s="24"/>
       <c r="M3" s="24"/>
       <c r="N3" s="24"/>
@@ -38182,11 +38176,11 @@
         <v>9</v>
       </c>
       <c r="F4" s="24"/>
-      <c r="G4" s="29"/>
-      <c r="H4" s="30"/>
-      <c r="I4" s="30"/>
-      <c r="J4" s="30"/>
-      <c r="K4" s="30"/>
+      <c r="G4" s="13"/>
+      <c r="H4" s="14"/>
+      <c r="I4" s="14"/>
+      <c r="J4" s="14"/>
+      <c r="K4" s="14"/>
       <c r="L4" s="24"/>
       <c r="M4" s="24"/>
       <c r="N4" s="24"/>
@@ -38196,8 +38190,8 @@
       <c r="R4" s="24"/>
     </row>
     <row r="5" spans="1:18" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A5" s="27" t="s">
-        <v>27</v>
+      <c r="A5" s="25" t="s">
+        <v>9</v>
       </c>
       <c r="B5" s="27" t="s">
         <v>82</v>
@@ -38212,11 +38206,11 @@
         <v>9</v>
       </c>
       <c r="F5" s="24"/>
-      <c r="G5" s="29"/>
-      <c r="H5" s="30"/>
-      <c r="I5" s="30"/>
-      <c r="J5" s="30"/>
-      <c r="K5" s="30"/>
+      <c r="G5" s="13"/>
+      <c r="H5" s="14"/>
+      <c r="I5" s="14"/>
+      <c r="J5" s="14"/>
+      <c r="K5" s="14"/>
       <c r="L5" s="24"/>
       <c r="M5" s="24"/>
       <c r="N5" s="24"/>
@@ -38226,8 +38220,8 @@
       <c r="R5" s="24"/>
     </row>
     <row r="6" spans="1:18" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A6" s="27" t="s">
-        <v>27</v>
+      <c r="A6" s="25" t="s">
+        <v>9</v>
       </c>
       <c r="B6" s="27" t="s">
         <v>83</v>
@@ -38238,15 +38232,15 @@
       <c r="D6" s="27" t="s">
         <v>106</v>
       </c>
-      <c r="E6" s="31" t="s">
+      <c r="E6" s="29" t="s">
         <v>27</v>
       </c>
       <c r="F6" s="24"/>
-      <c r="G6" s="29"/>
-      <c r="H6" s="30"/>
-      <c r="I6" s="30"/>
-      <c r="J6" s="30"/>
-      <c r="K6" s="30"/>
+      <c r="G6" s="13"/>
+      <c r="H6" s="14"/>
+      <c r="I6" s="14"/>
+      <c r="J6" s="14"/>
+      <c r="K6" s="14"/>
       <c r="L6" s="24"/>
       <c r="M6" s="24"/>
       <c r="N6" s="24"/>
@@ -38256,8 +38250,8 @@
       <c r="R6" s="24"/>
     </row>
     <row r="7" spans="1:18" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A7" s="27" t="s">
-        <v>27</v>
+      <c r="A7" s="25" t="s">
+        <v>9</v>
       </c>
       <c r="B7" s="27" t="s">
         <v>84</v>
@@ -38272,11 +38266,11 @@
         <v>9</v>
       </c>
       <c r="F7" s="24"/>
-      <c r="G7" s="29"/>
-      <c r="H7" s="30"/>
-      <c r="I7" s="30"/>
-      <c r="J7" s="30"/>
-      <c r="K7" s="30"/>
+      <c r="G7" s="13"/>
+      <c r="H7" s="14"/>
+      <c r="I7" s="14"/>
+      <c r="J7" s="14"/>
+      <c r="K7" s="14"/>
       <c r="L7" s="24"/>
       <c r="M7" s="24"/>
       <c r="N7" s="24"/>
@@ -38286,8 +38280,8 @@
       <c r="R7" s="24"/>
     </row>
     <row r="8" spans="1:18" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A8" s="27" t="s">
-        <v>27</v>
+      <c r="A8" s="25" t="s">
+        <v>9</v>
       </c>
       <c r="B8" s="27" t="s">
         <v>85</v>
@@ -38296,15 +38290,15 @@
       <c r="D8" s="27" t="s">
         <v>105</v>
       </c>
-      <c r="E8" s="31" t="s">
+      <c r="E8" s="29" t="s">
         <v>9</v>
       </c>
       <c r="F8" s="24"/>
-      <c r="G8" s="29"/>
-      <c r="H8" s="30"/>
-      <c r="I8" s="30"/>
-      <c r="J8" s="30"/>
-      <c r="K8" s="30"/>
+      <c r="G8" s="13"/>
+      <c r="H8" s="14"/>
+      <c r="I8" s="14"/>
+      <c r="J8" s="14"/>
+      <c r="K8" s="14"/>
       <c r="L8" s="24"/>
       <c r="M8" s="24"/>
       <c r="N8" s="24"/>
@@ -38314,8 +38308,8 @@
       <c r="R8" s="24"/>
     </row>
     <row r="9" spans="1:18" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A9" s="27" t="s">
-        <v>27</v>
+      <c r="A9" s="25" t="s">
+        <v>9</v>
       </c>
       <c r="B9" s="27" t="s">
         <v>86</v>
@@ -38326,15 +38320,15 @@
       <c r="D9" s="27" t="s">
         <v>106</v>
       </c>
-      <c r="E9" s="31" t="s">
+      <c r="E9" s="29" t="s">
         <v>27</v>
       </c>
       <c r="F9" s="24"/>
-      <c r="G9" s="29"/>
-      <c r="H9" s="30"/>
-      <c r="I9" s="30"/>
-      <c r="J9" s="30"/>
-      <c r="K9" s="30"/>
+      <c r="G9" s="13"/>
+      <c r="H9" s="14"/>
+      <c r="I9" s="14"/>
+      <c r="J9" s="14"/>
+      <c r="K9" s="14"/>
       <c r="L9" s="24"/>
       <c r="M9" s="24"/>
       <c r="N9" s="24"/>
@@ -38344,8 +38338,8 @@
       <c r="R9" s="24"/>
     </row>
     <row r="10" spans="1:18" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A10" s="27" t="s">
-        <v>27</v>
+      <c r="A10" s="25" t="s">
+        <v>9</v>
       </c>
       <c r="B10" s="27" t="s">
         <v>87</v>
@@ -38356,15 +38350,15 @@
       <c r="D10" s="27" t="s">
         <v>106</v>
       </c>
-      <c r="E10" s="31" t="s">
+      <c r="E10" s="29" t="s">
         <v>27</v>
       </c>
       <c r="F10" s="24"/>
-      <c r="G10" s="29"/>
-      <c r="H10" s="30"/>
-      <c r="I10" s="30"/>
-      <c r="J10" s="30"/>
-      <c r="K10" s="30"/>
+      <c r="G10" s="13"/>
+      <c r="H10" s="14"/>
+      <c r="I10" s="14"/>
+      <c r="J10" s="14"/>
+      <c r="K10" s="14"/>
       <c r="L10" s="24"/>
       <c r="M10" s="24"/>
       <c r="N10" s="24"/>

</xml_diff>